<commit_message>
Store decode token times as JSON string instead of mean value
Co-authored-by: liuruijin17 <liuruijin17@gmail.com>
</commit_message>
<xml_diff>
--- a/out.xlsx
+++ b/out.xlsx
@@ -483,8 +483,10 @@
       <c r="F2" t="n">
         <v>1087.249387986958</v>
       </c>
-      <c r="G2" t="n">
-        <v>270.110630164189</v>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>[1699.4226472452283, 31.91912453621626, 31.829772517085075, 31.765862368047237, 32.48662035912275, 31.398748978972435, 31.951635144650936]</t>
+        </is>
       </c>
       <c r="H2" t="n">
         <v>2.978405034169555</v>

</xml_diff>